<commit_message>
Expand system_init.xlsx for meetings/decisions/comments/links
</commit_message>
<xml_diff>
--- a/src/main/resources/excel/system_init_min.xlsx
+++ b/src/main/resources/excel/system_init_min.xlsx
@@ -12,14 +12,16 @@
     <sheet name="Activity Priority" r:id="rId6" sheetId="4"/>
     <sheet name="Activity Type" r:id="rId7" sheetId="5"/>
     <sheet name="Issue Type" r:id="rId8" sheetId="6"/>
-    <sheet name="Grid Entity" r:id="rId9" sheetId="7"/>
-    <sheet name="Page Entity" r:id="rId10" sheetId="8"/>
+    <sheet name="Meeting Type" r:id="rId9" sheetId="7"/>
+    <sheet name="Decision Type" r:id="rId10" sheetId="8"/>
+    <sheet name="Grid Entity" r:id="rId11" sheetId="9"/>
+    <sheet name="Page Entity" r:id="rId12" sheetId="10"/>
   </sheets>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="186" uniqueCount="100">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="261" uniqueCount="113">
   <si>
     <t># Project Item Statuses (used by Activities, Issues, etc.)</t>
   </si>
@@ -72,6 +74,9 @@
     <t># Columns: Name (required)</t>
   </si>
   <si>
+    <t>Agile Item Workflow</t>
+  </si>
+  <si>
     <t>Default Workflow</t>
   </si>
   <si>
@@ -217,6 +222,42 @@
   </si>
   <si>
     <t>#7B1FA2</t>
+  </si>
+  <si>
+    <t># Meeting Types</t>
+  </si>
+  <si>
+    <t>Sprint Planning</t>
+  </si>
+  <si>
+    <t>#DAA520</t>
+  </si>
+  <si>
+    <t>Sprint Retrospective</t>
+  </si>
+  <si>
+    <t>Project Review</t>
+  </si>
+  <si>
+    <t># Decision Types</t>
+  </si>
+  <si>
+    <t># Columns: Name (required), Color, Sort Order, Level, Can Have Children, Non Deletable, Workflow, Requires Approval</t>
+  </si>
+  <si>
+    <t>Requires Approval</t>
+  </si>
+  <si>
+    <t>Technical</t>
+  </si>
+  <si>
+    <t>#91856C</t>
+  </si>
+  <si>
+    <t>Strategic</t>
+  </si>
+  <si>
+    <t>Budget</t>
   </si>
   <si>
     <t># Grid Entities (view configuration)</t>
@@ -326,13 +367,37 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="17">
+  <fonts count="21">
     <font>
       <sz val="11.0"/>
       <color indexed="8"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <b val="true"/>
+      <color indexed="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <i val="true"/>
+      <color indexed="23"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <b val="true"/>
+      <color indexed="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <i val="true"/>
+      <color indexed="23"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -464,7 +529,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="true" applyFill="true" applyBorder="true"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="true"/>
@@ -482,6 +547,10 @@
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true"/>
     <xf numFmtId="0" fontId="15" fillId="3" borderId="1" xfId="0" applyFont="true" applyFill="true" applyBorder="true"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true"/>
+    <xf numFmtId="0" fontId="17" fillId="3" borderId="1" xfId="0" applyFont="true" applyFill="true" applyBorder="true"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="true"/>
+    <xf numFmtId="0" fontId="19" fillId="3" borderId="1" xfId="0" applyFont="true" applyFill="true" applyBorder="true"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="true"/>
   </cellXfs>
 </styleSheet>
 </file>
@@ -568,9 +637,127 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:I5"/>
+  <sheetFormatPr defaultRowHeight="15.0"/>
+  <cols>
+    <col min="1" max="1" width="92.71484375" customWidth="true" bestFit="true"/>
+    <col min="2" max="2" width="20.0859375" customWidth="true" bestFit="true"/>
+    <col min="3" max="3" width="11.48828125" customWidth="true" bestFit="true"/>
+    <col min="4" max="4" width="13.875" customWidth="true" bestFit="true"/>
+    <col min="5" max="5" width="17.8515625" customWidth="true" bestFit="true"/>
+    <col min="6" max="6" width="11.05859375" customWidth="true" bestFit="true"/>
+    <col min="7" max="7" width="22.27734375" customWidth="true" bestFit="true"/>
+    <col min="8" max="8" width="12.171875" customWidth="true" bestFit="true"/>
+    <col min="9" max="9" width="7.98046875" customWidth="true" bestFit="true"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s" s="20">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s" s="20">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s" s="19">
+        <v>2</v>
+      </c>
+      <c r="B3" t="s" s="19">
+        <v>94</v>
+      </c>
+      <c r="C3" t="s" s="19">
+        <v>95</v>
+      </c>
+      <c r="D3" t="s" s="19">
+        <v>96</v>
+      </c>
+      <c r="E3" t="s" s="19">
+        <v>97</v>
+      </c>
+      <c r="F3" t="s" s="19">
+        <v>5</v>
+      </c>
+      <c r="G3" t="s" s="19">
+        <v>98</v>
+      </c>
+      <c r="H3" t="s" s="19">
+        <v>99</v>
+      </c>
+      <c r="I3" t="s" s="19">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s" s="0">
+        <v>101</v>
+      </c>
+      <c r="B4" t="s" s="0">
+        <v>102</v>
+      </c>
+      <c r="C4" t="s" s="0">
+        <v>103</v>
+      </c>
+      <c r="D4" t="s" s="0">
+        <v>104</v>
+      </c>
+      <c r="E4" t="s" s="0">
+        <v>105</v>
+      </c>
+      <c r="F4" t="s" s="0">
+        <v>106</v>
+      </c>
+      <c r="G4" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="H4" t="s" s="0">
+        <v>85</v>
+      </c>
+      <c r="I4" t="s" s="0">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s" s="0">
+        <v>107</v>
+      </c>
+      <c r="B5" t="s" s="0">
+        <v>108</v>
+      </c>
+      <c r="C5" t="s" s="0">
+        <v>109</v>
+      </c>
+      <c r="D5" t="s" s="0">
+        <v>110</v>
+      </c>
+      <c r="E5" t="s" s="0">
+        <v>111</v>
+      </c>
+      <c r="F5" t="s" s="0">
+        <v>112</v>
+      </c>
+      <c r="G5" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="H5" t="s" s="0">
+        <v>89</v>
+      </c>
+      <c r="I5" t="s" s="0">
+        <v>26</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:A4"/>
+  <dimension ref="A1:A5"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="22.9140625" customWidth="true" bestFit="true"/>
@@ -596,6 +783,11 @@
         <v>17</v>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="s" s="0">
+        <v>18</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
@@ -603,7 +795,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="81.234375" customWidth="true" bestFit="true"/>
@@ -615,29 +807,29 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s" s="6">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s" s="6">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s" s="5">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B3" t="s" s="5">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C3" t="s" s="5">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D3" t="s" s="5">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E3" t="s" s="5">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="4">
@@ -654,7 +846,7 @@
         <v>13</v>
       </c>
       <c r="E4" t="s" s="0">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="5">
@@ -671,7 +863,41 @@
         <v>7</v>
       </c>
       <c r="E5" t="s" s="0">
-        <v>25</v>
+        <v>26</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s" s="0">
+        <v>18</v>
+      </c>
+      <c r="B6" t="s" s="0">
+        <v>6</v>
+      </c>
+      <c r="C6" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="D6" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="E6" t="s" s="0">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s" s="0">
+        <v>18</v>
+      </c>
+      <c r="B7" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="C7" t="s" s="0">
+        <v>12</v>
+      </c>
+      <c r="D7" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="E7" t="s" s="0">
+        <v>26</v>
       </c>
     </row>
   </sheetData>
@@ -693,12 +919,12 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s" s="8">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s" s="8">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="3">
@@ -709,27 +935,27 @@
         <v>4</v>
       </c>
       <c r="C3" t="s" s="7">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D3" t="s" s="7">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="E3" t="s" s="7">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s" s="0">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B4" t="s" s="0">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C4" t="s" s="0">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D4" t="s" s="0">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="E4" t="s" s="0">
         <v>7</v>
@@ -737,16 +963,16 @@
     </row>
     <row r="5">
       <c r="A5" t="s" s="0">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B5" t="s" s="0">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C5" t="s" s="0">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D5" t="s" s="0">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="E5" t="s" s="0">
         <v>7</v>
@@ -754,16 +980,16 @@
     </row>
     <row r="6">
       <c r="A6" t="s" s="0">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B6" t="s" s="0">
         <v>11</v>
       </c>
       <c r="C6" t="s" s="0">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D6" t="s" s="0">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E6" t="s" s="0">
         <v>13</v>
@@ -771,16 +997,16 @@
     </row>
     <row r="7">
       <c r="A7" t="s" s="0">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B7" t="s" s="0">
         <v>8</v>
       </c>
       <c r="C7" t="s" s="0">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="D7" t="s" s="0">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E7" t="s" s="0">
         <v>7</v>
@@ -802,17 +1028,17 @@
     <col min="4" max="4" width="5.51953125" customWidth="true" bestFit="true"/>
     <col min="5" max="5" width="16.99609375" customWidth="true" bestFit="true"/>
     <col min="6" max="6" width="13.42578125" customWidth="true" bestFit="true"/>
-    <col min="7" max="7" width="15.19921875" customWidth="true" bestFit="true"/>
+    <col min="7" max="7" width="17.5703125" customWidth="true" bestFit="true"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="s" s="10">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s" s="10">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="3">
@@ -823,33 +1049,33 @@
         <v>4</v>
       </c>
       <c r="C3" t="s" s="9">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D3" t="s" s="9">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="E3" t="s" s="9">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="F3" t="s" s="9">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="G3" t="s" s="9">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s" s="0">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B4" t="s" s="0">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C4" t="s" s="0">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D4" t="s" s="0">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="E4" t="s" s="0">
         <v>7</v>
@@ -863,16 +1089,16 @@
     </row>
     <row r="5">
       <c r="A5" t="s" s="0">
+        <v>54</v>
+      </c>
+      <c r="B5" t="s" s="0">
+        <v>55</v>
+      </c>
+      <c r="C5" t="s" s="0">
+        <v>38</v>
+      </c>
+      <c r="D5" t="s" s="0">
         <v>53</v>
-      </c>
-      <c r="B5" t="s" s="0">
-        <v>54</v>
-      </c>
-      <c r="C5" t="s" s="0">
-        <v>37</v>
-      </c>
-      <c r="D5" t="s" s="0">
-        <v>52</v>
       </c>
       <c r="E5" t="s" s="0">
         <v>7</v>
@@ -886,16 +1112,16 @@
     </row>
     <row r="6">
       <c r="A6" t="s" s="0">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B6" t="s" s="0">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C6" t="s" s="0">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D6" t="s" s="0">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="E6" t="s" s="0">
         <v>7</v>
@@ -909,16 +1135,16 @@
     </row>
     <row r="7">
       <c r="A7" t="s" s="0">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B7" t="s" s="0">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C7" t="s" s="0">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="D7" t="s" s="0">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="E7" t="s" s="0">
         <v>7</v>
@@ -946,17 +1172,17 @@
     <col min="4" max="4" width="5.51953125" customWidth="true" bestFit="true"/>
     <col min="5" max="5" width="16.99609375" customWidth="true" bestFit="true"/>
     <col min="6" max="6" width="13.42578125" customWidth="true" bestFit="true"/>
-    <col min="7" max="7" width="15.19921875" customWidth="true" bestFit="true"/>
+    <col min="7" max="7" width="17.5703125" customWidth="true" bestFit="true"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="s" s="12">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s" s="12">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="3">
@@ -967,33 +1193,33 @@
         <v>4</v>
       </c>
       <c r="C3" t="s" s="11">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D3" t="s" s="11">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="E3" t="s" s="11">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="F3" t="s" s="11">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="G3" t="s" s="11">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s" s="0">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B4" t="s" s="0">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C4" t="s" s="0">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D4" t="s" s="0">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="E4" t="s" s="0">
         <v>7</v>
@@ -1007,16 +1233,16 @@
     </row>
     <row r="5">
       <c r="A5" t="s" s="0">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B5" t="s" s="0">
         <v>8</v>
       </c>
       <c r="C5" t="s" s="0">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D5" t="s" s="0">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="E5" t="s" s="0">
         <v>7</v>
@@ -1030,16 +1256,16 @@
     </row>
     <row r="6">
       <c r="A6" t="s" s="0">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B6" t="s" s="0">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="C6" t="s" s="0">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D6" t="s" s="0">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="E6" t="s" s="0">
         <v>7</v>
@@ -1053,16 +1279,16 @@
     </row>
     <row r="7">
       <c r="A7" t="s" s="0">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B7" t="s" s="0">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C7" t="s" s="0">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="D7" t="s" s="0">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="E7" t="s" s="0">
         <v>7</v>
@@ -1080,6 +1306,261 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:G6"/>
+  <sheetFormatPr defaultRowHeight="15.0"/>
+  <cols>
+    <col min="1" max="1" width="77.05078125" customWidth="true" bestFit="true"/>
+    <col min="2" max="2" width="8.5546875" customWidth="true" bestFit="true"/>
+    <col min="3" max="3" width="10.109375" customWidth="true" bestFit="true"/>
+    <col min="4" max="4" width="5.51953125" customWidth="true" bestFit="true"/>
+    <col min="5" max="5" width="16.99609375" customWidth="true" bestFit="true"/>
+    <col min="6" max="6" width="13.42578125" customWidth="true" bestFit="true"/>
+    <col min="7" max="7" width="17.5703125" customWidth="true" bestFit="true"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s" s="14">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s" s="14">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s" s="13">
+        <v>2</v>
+      </c>
+      <c r="B3" t="s" s="13">
+        <v>4</v>
+      </c>
+      <c r="C3" t="s" s="13">
+        <v>29</v>
+      </c>
+      <c r="D3" t="s" s="13">
+        <v>48</v>
+      </c>
+      <c r="E3" t="s" s="13">
+        <v>49</v>
+      </c>
+      <c r="F3" t="s" s="13">
+        <v>50</v>
+      </c>
+      <c r="G3" t="s" s="13">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s" s="0">
+        <v>68</v>
+      </c>
+      <c r="B4" t="s" s="0">
+        <v>69</v>
+      </c>
+      <c r="C4" t="s" s="0">
+        <v>34</v>
+      </c>
+      <c r="D4" t="s" s="0">
+        <v>53</v>
+      </c>
+      <c r="E4" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="F4" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="G4" t="s" s="0">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s" s="0">
+        <v>70</v>
+      </c>
+      <c r="B5" t="s" s="0">
+        <v>69</v>
+      </c>
+      <c r="C5" t="s" s="0">
+        <v>38</v>
+      </c>
+      <c r="D5" t="s" s="0">
+        <v>53</v>
+      </c>
+      <c r="E5" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="F5" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="G5" t="s" s="0">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s" s="0">
+        <v>71</v>
+      </c>
+      <c r="B6" t="s" s="0">
+        <v>69</v>
+      </c>
+      <c r="C6" t="s" s="0">
+        <v>41</v>
+      </c>
+      <c r="D6" t="s" s="0">
+        <v>53</v>
+      </c>
+      <c r="E6" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="F6" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="G6" t="s" s="0">
+        <v>17</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:H6"/>
+  <sheetFormatPr defaultRowHeight="15.0"/>
+  <cols>
+    <col min="1" max="1" width="92.02734375" customWidth="true" bestFit="true"/>
+    <col min="2" max="2" width="8.1484375" customWidth="true" bestFit="true"/>
+    <col min="3" max="3" width="10.109375" customWidth="true" bestFit="true"/>
+    <col min="4" max="4" width="5.51953125" customWidth="true" bestFit="true"/>
+    <col min="5" max="5" width="16.99609375" customWidth="true" bestFit="true"/>
+    <col min="6" max="6" width="13.42578125" customWidth="true" bestFit="true"/>
+    <col min="7" max="7" width="17.5703125" customWidth="true" bestFit="true"/>
+    <col min="8" max="8" width="16.94140625" customWidth="true" bestFit="true"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s" s="16">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s" s="16">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s" s="15">
+        <v>2</v>
+      </c>
+      <c r="B3" t="s" s="15">
+        <v>4</v>
+      </c>
+      <c r="C3" t="s" s="15">
+        <v>29</v>
+      </c>
+      <c r="D3" t="s" s="15">
+        <v>48</v>
+      </c>
+      <c r="E3" t="s" s="15">
+        <v>49</v>
+      </c>
+      <c r="F3" t="s" s="15">
+        <v>50</v>
+      </c>
+      <c r="G3" t="s" s="15">
+        <v>21</v>
+      </c>
+      <c r="H3" t="s" s="15">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s" s="0">
+        <v>75</v>
+      </c>
+      <c r="B4" t="s" s="0">
+        <v>76</v>
+      </c>
+      <c r="C4" t="s" s="0">
+        <v>34</v>
+      </c>
+      <c r="D4" t="s" s="0">
+        <v>53</v>
+      </c>
+      <c r="E4" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="F4" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="G4" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="H4" t="s" s="0">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s" s="0">
+        <v>77</v>
+      </c>
+      <c r="B5" t="s" s="0">
+        <v>76</v>
+      </c>
+      <c r="C5" t="s" s="0">
+        <v>38</v>
+      </c>
+      <c r="D5" t="s" s="0">
+        <v>53</v>
+      </c>
+      <c r="E5" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="F5" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="G5" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="H5" t="s" s="0">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s" s="0">
+        <v>78</v>
+      </c>
+      <c r="B6" t="s" s="0">
+        <v>76</v>
+      </c>
+      <c r="C6" t="s" s="0">
+        <v>41</v>
+      </c>
+      <c r="D6" t="s" s="0">
+        <v>53</v>
+      </c>
+      <c r="E6" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="F6" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="G6" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="H6" t="s" s="0">
+        <v>13</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <dimension ref="A1:E5"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
@@ -1092,44 +1573,44 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="s" s="14">
-        <v>66</v>
+      <c r="A1" t="s" s="18">
+        <v>79</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="s" s="14">
-        <v>67</v>
+      <c r="A2" t="s" s="18">
+        <v>80</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="s" s="13">
+      <c r="A3" t="s" s="17">
         <v>2</v>
       </c>
-      <c r="B3" t="s" s="13">
-        <v>68</v>
-      </c>
-      <c r="C3" t="s" s="13">
-        <v>69</v>
-      </c>
-      <c r="D3" t="s" s="13">
-        <v>70</v>
-      </c>
-      <c r="E3" t="s" s="13">
-        <v>71</v>
+      <c r="B3" t="s" s="17">
+        <v>81</v>
+      </c>
+      <c r="C3" t="s" s="17">
+        <v>82</v>
+      </c>
+      <c r="D3" t="s" s="17">
+        <v>83</v>
+      </c>
+      <c r="E3" t="s" s="17">
+        <v>84</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s" s="0">
-        <v>72</v>
+        <v>85</v>
       </c>
       <c r="B4" t="s" s="0">
-        <v>73</v>
+        <v>86</v>
       </c>
       <c r="C4" t="s" s="0">
-        <v>74</v>
+        <v>87</v>
       </c>
       <c r="D4" t="s" s="0">
-        <v>75</v>
+        <v>88</v>
       </c>
       <c r="E4" t="s" s="0">
         <v>7</v>
@@ -1137,137 +1618,19 @@
     </row>
     <row r="5">
       <c r="A5" t="s" s="0">
-        <v>76</v>
+        <v>89</v>
       </c>
       <c r="B5" t="s" s="0">
-        <v>77</v>
+        <v>90</v>
       </c>
       <c r="C5" t="s" s="0">
-        <v>78</v>
+        <v>91</v>
       </c>
       <c r="D5" t="s" s="0">
-        <v>75</v>
+        <v>88</v>
       </c>
       <c r="E5" t="s" s="0">
         <v>7</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:I5"/>
-  <sheetFormatPr defaultRowHeight="15.0"/>
-  <cols>
-    <col min="1" max="1" width="92.71484375" customWidth="true" bestFit="true"/>
-    <col min="2" max="2" width="20.0859375" customWidth="true" bestFit="true"/>
-    <col min="3" max="3" width="11.48828125" customWidth="true" bestFit="true"/>
-    <col min="4" max="4" width="13.875" customWidth="true" bestFit="true"/>
-    <col min="5" max="5" width="17.8515625" customWidth="true" bestFit="true"/>
-    <col min="6" max="6" width="11.05859375" customWidth="true" bestFit="true"/>
-    <col min="7" max="7" width="22.27734375" customWidth="true" bestFit="true"/>
-    <col min="8" max="8" width="12.171875" customWidth="true" bestFit="true"/>
-    <col min="9" max="9" width="7.98046875" customWidth="true" bestFit="true"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="s" s="16">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="s" s="16">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="s" s="15">
-        <v>2</v>
-      </c>
-      <c r="B3" t="s" s="15">
-        <v>81</v>
-      </c>
-      <c r="C3" t="s" s="15">
-        <v>82</v>
-      </c>
-      <c r="D3" t="s" s="15">
-        <v>83</v>
-      </c>
-      <c r="E3" t="s" s="15">
-        <v>84</v>
-      </c>
-      <c r="F3" t="s" s="15">
-        <v>5</v>
-      </c>
-      <c r="G3" t="s" s="15">
-        <v>85</v>
-      </c>
-      <c r="H3" t="s" s="15">
-        <v>86</v>
-      </c>
-      <c r="I3" t="s" s="15">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="s" s="0">
-        <v>88</v>
-      </c>
-      <c r="B4" t="s" s="0">
-        <v>89</v>
-      </c>
-      <c r="C4" t="s" s="0">
-        <v>90</v>
-      </c>
-      <c r="D4" t="s" s="0">
-        <v>91</v>
-      </c>
-      <c r="E4" t="s" s="0">
-        <v>92</v>
-      </c>
-      <c r="F4" t="s" s="0">
-        <v>93</v>
-      </c>
-      <c r="G4" t="s" s="0">
-        <v>13</v>
-      </c>
-      <c r="H4" t="s" s="0">
-        <v>72</v>
-      </c>
-      <c r="I4" t="s" s="0">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="s" s="0">
-        <v>94</v>
-      </c>
-      <c r="B5" t="s" s="0">
-        <v>95</v>
-      </c>
-      <c r="C5" t="s" s="0">
-        <v>96</v>
-      </c>
-      <c r="D5" t="s" s="0">
-        <v>97</v>
-      </c>
-      <c r="E5" t="s" s="0">
-        <v>98</v>
-      </c>
-      <c r="F5" t="s" s="0">
-        <v>99</v>
-      </c>
-      <c r="G5" t="s" s="0">
-        <v>13</v>
-      </c>
-      <c r="H5" t="s" s="0">
-        <v>76</v>
-      </c>
-      <c r="I5" t="s" s="0">
-        <v>25</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Refactor import handlers to utilize applyMetaFieldsDeclaredOn for field mapping
</commit_message>
<xml_diff>
--- a/src/main/resources/excel/system_init_min.xlsx
+++ b/src/main/resources/excel/system_init_min.xlsx
@@ -1,29 +1,29 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Workflow Entity" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Workflow Status Relation" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Activity Priority" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Activity Type" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Issue Type" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Meeting Type" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decision Type" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Epic Type" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Type" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="User Story Type" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirement Type" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Milestone Type" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Deliverable Type" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint Type" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ticket Priority" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ticket Type" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet name="Status" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Workflow Entity" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Workflow Status Relation" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Activity Priority" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Activity Type" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Issue Type" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Meeting Type" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Decision Type" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Epic Type" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Feature Type" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="User Story Type" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Requirement Type" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="Milestone Type" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="Deliverable Type" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="Sprint Type" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="Ticket Priority" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="Ticket Type" sheetId="17" state="visible" r:id="rId17"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -489,7 +489,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Derbent</t>
+          <t>Of Teknoloji Çözümleri</t>
         </is>
       </c>
     </row>
@@ -516,7 +516,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Derbent</t>
+          <t>Of Teknoloji Çözümleri</t>
         </is>
       </c>
     </row>
@@ -543,7 +543,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Derbent</t>
+          <t>Of Teknoloji Çözümleri</t>
         </is>
       </c>
     </row>
@@ -648,7 +648,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Derbent</t>
+          <t>Of Teknoloji Çözümleri</t>
         </is>
       </c>
     </row>
@@ -753,7 +753,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Derbent</t>
+          <t>Of Teknoloji Çözümleri</t>
         </is>
       </c>
     </row>
@@ -858,7 +858,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Derbent</t>
+          <t>Of Teknoloji Çözümleri</t>
         </is>
       </c>
     </row>
@@ -963,7 +963,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Derbent</t>
+          <t>Of Teknoloji Çözümleri</t>
         </is>
       </c>
     </row>
@@ -1068,7 +1068,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Derbent</t>
+          <t>Of Teknoloji Çözümleri</t>
         </is>
       </c>
     </row>
@@ -1173,7 +1173,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Derbent</t>
+          <t>Of Teknoloji Çözümleri</t>
         </is>
       </c>
     </row>
@@ -1258,7 +1258,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Derbent</t>
+          <t>Of Teknoloji Çözümleri</t>
         </is>
       </c>
     </row>
@@ -1363,7 +1363,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Derbent</t>
+          <t>Of Teknoloji Çözümleri</t>
         </is>
       </c>
     </row>
@@ -1408,7 +1408,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Derbent</t>
+          <t>Of Teknoloji Çözümleri</t>
         </is>
       </c>
     </row>
@@ -1420,7 +1420,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Derbent</t>
+          <t>Of Teknoloji Çözümleri</t>
         </is>
       </c>
     </row>
@@ -1498,10 +1498,9 @@
           <t>true</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Derbent</t>
+          <t>Of Teknoloji Çözümleri</t>
         </is>
       </c>
     </row>
@@ -1526,10 +1525,9 @@
           <t>false</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Derbent</t>
+          <t>Of Teknoloji Çözümleri</t>
         </is>
       </c>
     </row>
@@ -1554,10 +1552,9 @@
           <t>true</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Derbent</t>
+          <t>Of Teknoloji Çözümleri</t>
         </is>
       </c>
     </row>
@@ -1582,10 +1579,9 @@
           <t>false</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Derbent</t>
+          <t>Of Teknoloji Çözümleri</t>
         </is>
       </c>
     </row>
@@ -1670,7 +1666,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Derbent</t>
+          <t>Of Teknoloji Çözümleri</t>
         </is>
       </c>
     </row>
@@ -1702,7 +1698,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Derbent</t>
+          <t>Of Teknoloji Çözümleri</t>
         </is>
       </c>
     </row>
@@ -1807,7 +1803,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Derbent</t>
+          <t>Of Teknoloji Çözümleri</t>
         </is>
       </c>
     </row>
@@ -1912,7 +1908,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Derbent</t>
+          <t>Of Teknoloji Çözümleri</t>
         </is>
       </c>
     </row>
@@ -2017,7 +2013,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Derbent</t>
+          <t>Of Teknoloji Çözümleri</t>
         </is>
       </c>
     </row>
@@ -2132,7 +2128,7 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Derbent</t>
+          <t>Of Teknoloji Çözümleri</t>
         </is>
       </c>
     </row>
@@ -2237,7 +2233,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Derbent</t>
+          <t>Of Teknoloji Çözümleri</t>
         </is>
       </c>
     </row>

</xml_diff>